<commit_message>
ReadRootfile MC + ReadRootfile
</commit_message>
<xml_diff>
--- a/Belle2/data.xlsx
+++ b/Belle2/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\purol\OneDrive\바탕 화면\github\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26BB4799-6532-474B-BA13-09DA0CDC4F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D121037-724B-4908-BB7D-0B2D0A426BEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -349,22 +349,22 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A1">
-        <v>0.71235400000000004</v>
+        <v>0.81627099999999997</v>
       </c>
       <c r="B1">
-        <v>0.20435400000000001</v>
+        <v>0.150508</v>
       </c>
       <c r="C1">
-        <v>5.7730000000000004E-3</v>
+        <v>3.3899999999999998E-3</v>
       </c>
       <c r="D1">
-        <v>1.8140000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="E1">
-        <v>6.6E-4</v>
+        <v>0</v>
       </c>
       <c r="F1">
-        <v>1.3190000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="G1">
         <v>0</v>
@@ -379,16 +379,16 @@
         <v>0</v>
       </c>
       <c r="K1">
-        <v>1.65E-4</v>
+        <v>0</v>
       </c>
       <c r="L1">
-        <v>3.1503000000000003E-2</v>
+        <v>1.3559E-2</v>
       </c>
       <c r="M1">
-        <v>1.65E-4</v>
+        <v>0</v>
       </c>
       <c r="N1">
-        <v>4.4530000000000004E-3</v>
+        <v>6.78E-4</v>
       </c>
       <c r="O1">
         <v>0</v>
@@ -406,33 +406,33 @@
         <v>0</v>
       </c>
       <c r="T1">
-        <v>1.65E-4</v>
+        <v>0</v>
       </c>
       <c r="U1">
-        <v>3.7275000000000003E-2</v>
+        <v>1.5592999999999999E-2</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A2">
-        <v>4.0670999999999999E-2</v>
+        <v>5.5275999999999999E-2</v>
       </c>
       <c r="B2">
-        <v>0.773289</v>
+        <v>0.78391999999999995</v>
       </c>
       <c r="C2">
-        <v>6.0460000000000002E-3</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>1.9239999999999999E-3</v>
+        <v>2.513E-3</v>
       </c>
       <c r="E2">
-        <v>5.7710000000000001E-3</v>
+        <v>1.005E-2</v>
       </c>
       <c r="F2">
-        <v>6.3200000000000001E-3</v>
+        <v>2.513E-3</v>
       </c>
       <c r="G2">
-        <v>2.7500000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -447,25 +447,25 @@
         <v>0</v>
       </c>
       <c r="L2">
-        <v>1.1816E-2</v>
+        <v>1.5075E-2</v>
       </c>
       <c r="M2">
-        <v>1.0989999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <v>2.061E-2</v>
+        <v>7.5380000000000004E-3</v>
       </c>
       <c r="O2">
-        <v>2.7500000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="P2">
         <v>0</v>
       </c>
       <c r="Q2">
-        <v>8.2399999999999997E-4</v>
+        <v>0</v>
       </c>
       <c r="R2">
-        <v>2.7500000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="S2">
         <v>0</v>
@@ -474,30 +474,30 @@
         <v>0</v>
       </c>
       <c r="U2">
-        <v>0.130805</v>
+        <v>0.123116</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A3">
-        <v>5.1000000000000004E-4</v>
+        <v>3.5839999999999999E-3</v>
       </c>
       <c r="B3">
         <v>0</v>
       </c>
       <c r="C3">
-        <v>0.82763900000000001</v>
+        <v>0.92114700000000005</v>
       </c>
       <c r="D3">
-        <v>2.0400000000000001E-3</v>
+        <v>3.5839999999999999E-3</v>
       </c>
       <c r="E3">
-        <v>0.11677700000000001</v>
+        <v>6.0932E-2</v>
       </c>
       <c r="F3">
-        <v>5.1000000000000004E-4</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>1.5299999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -509,25 +509,25 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>5.6090000000000003E-3</v>
+        <v>7.1679999999999999E-3</v>
       </c>
       <c r="L3">
-        <v>5.1000000000000004E-4</v>
+        <v>0</v>
       </c>
       <c r="M3">
-        <v>7.6490000000000004E-3</v>
+        <v>0</v>
       </c>
       <c r="N3">
         <v>0</v>
       </c>
       <c r="O3">
-        <v>8.6689999999999996E-3</v>
+        <v>3.5839999999999999E-3</v>
       </c>
       <c r="P3">
         <v>0</v>
       </c>
       <c r="Q3">
-        <v>5.6090000000000003E-3</v>
+        <v>0</v>
       </c>
       <c r="R3">
         <v>0</v>
@@ -539,60 +539,60 @@
         <v>0</v>
       </c>
       <c r="U3">
-        <v>2.2946999999999999E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A4">
-        <v>6.0099999999999997E-4</v>
+        <v>0</v>
       </c>
       <c r="B4">
-        <v>4.8079999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="C4">
-        <v>9.0139999999999994E-3</v>
+        <v>1.5873000000000002E-2</v>
       </c>
       <c r="D4">
-        <v>0.579928</v>
+        <v>0.730159</v>
       </c>
       <c r="E4">
-        <v>1.2019999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>0.241587</v>
+        <v>0.19047600000000001</v>
       </c>
       <c r="G4">
-        <v>3.6059999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>6.0099999999999997E-4</v>
+        <v>5.2909999999999997E-3</v>
       </c>
       <c r="I4">
-        <v>1.2019999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>6.0099999999999997E-4</v>
+        <v>0</v>
       </c>
       <c r="K4">
-        <v>1.2019999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="L4">
-        <v>2.8846E-2</v>
+        <v>1.5873000000000002E-2</v>
       </c>
       <c r="M4">
         <v>0</v>
       </c>
       <c r="N4">
-        <v>2.1635000000000001E-2</v>
+        <v>1.0581999999999999E-2</v>
       </c>
       <c r="O4">
-        <v>6.0099999999999997E-4</v>
+        <v>0</v>
       </c>
       <c r="P4">
-        <v>1.4423E-2</v>
+        <v>5.2909999999999997E-3</v>
       </c>
       <c r="Q4">
-        <v>6.0099999999999997E-4</v>
+        <v>0</v>
       </c>
       <c r="R4">
         <v>0</v>
@@ -604,7 +604,7 @@
         <v>0</v>
       </c>
       <c r="U4">
-        <v>8.9542999999999998E-2</v>
+        <v>2.6454999999999999E-2</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.45">
@@ -615,19 +615,19 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>0.19806799999999999</v>
+        <v>0.25</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>0.57246399999999997</v>
+        <v>0.5625</v>
       </c>
       <c r="F5">
-        <v>2.415E-3</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>2.415E-3</v>
+        <v>0</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -639,25 +639,25 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>2.415E-3</v>
+        <v>0</v>
       </c>
       <c r="L5">
         <v>0</v>
       </c>
       <c r="M5">
-        <v>1.4493000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="N5">
-        <v>2.415E-3</v>
+        <v>0</v>
       </c>
       <c r="O5">
-        <v>2.4154999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="P5">
         <v>0</v>
       </c>
       <c r="Q5">
-        <v>1.6907999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="R5">
         <v>0</v>
@@ -669,7 +669,7 @@
         <v>0</v>
       </c>
       <c r="U5">
-        <v>0.16425100000000001</v>
+        <v>0.1875</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.45">
@@ -677,19 +677,19 @@
         <v>0</v>
       </c>
       <c r="B6">
-        <v>4.7060000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6">
-        <v>7.0587999999999998E-2</v>
+        <v>0.111111</v>
       </c>
       <c r="E6">
-        <v>2.3530000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="F6">
-        <v>0.55529399999999995</v>
+        <v>0.61111099999999996</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -707,22 +707,22 @@
         <v>0</v>
       </c>
       <c r="L6">
-        <v>1.1764999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="M6">
         <v>0</v>
       </c>
       <c r="N6">
-        <v>2.8235E-2</v>
+        <v>0</v>
       </c>
       <c r="O6">
-        <v>2.3530000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>7.0590000000000002E-3</v>
+        <v>0</v>
       </c>
       <c r="Q6">
-        <v>2.3530000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="R6">
         <v>0</v>
@@ -734,7 +734,7 @@
         <v>0</v>
       </c>
       <c r="U6">
-        <v>0.31529400000000002</v>
+        <v>0.27777800000000002</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.45">
@@ -745,19 +745,19 @@
         <v>0</v>
       </c>
       <c r="C7">
-        <v>1.5625E-2</v>
+        <v>0</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>1.5625E-2</v>
+        <v>0</v>
       </c>
       <c r="F7">
         <v>0</v>
       </c>
       <c r="G7">
-        <v>0.328125</v>
+        <v>0.33333299999999999</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -778,16 +778,16 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <v>1.5625E-2</v>
+        <v>0</v>
       </c>
       <c r="O7">
-        <v>1.5625E-2</v>
+        <v>0</v>
       </c>
       <c r="P7">
         <v>0</v>
       </c>
       <c r="Q7">
-        <v>9.375E-2</v>
+        <v>0</v>
       </c>
       <c r="R7">
         <v>0</v>
@@ -799,7 +799,7 @@
         <v>0</v>
       </c>
       <c r="U7">
-        <v>0.515625</v>
+        <v>0.66666700000000001</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.45">
@@ -807,31 +807,31 @@
         <v>0</v>
       </c>
       <c r="B8">
-        <v>1.1110999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
       <c r="D8">
-        <v>2.2221999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
       <c r="F8">
-        <v>1.1110999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8">
-        <v>8.8888999999999996E-2</v>
+        <v>0</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -858,13 +858,13 @@
         <v>0</v>
       </c>
       <c r="S8">
-        <v>4.4443999999999997E-2</v>
+        <v>0</v>
       </c>
       <c r="T8">
         <v>0</v>
       </c>
       <c r="U8">
-        <v>2.2221999999999999E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.45">
@@ -893,7 +893,7 @@
         <v>0</v>
       </c>
       <c r="I9">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -929,7 +929,7 @@
         <v>0</v>
       </c>
       <c r="U9">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.45">
@@ -955,13 +955,13 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>0.14285700000000001</v>
+        <v>0</v>
       </c>
       <c r="I10">
         <v>0</v>
       </c>
       <c r="J10">
-        <v>0.71428599999999998</v>
+        <v>0</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -994,7 +994,7 @@
         <v>0</v>
       </c>
       <c r="U10">
-        <v>0.14285700000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.45">
@@ -1005,13 +1005,13 @@
         <v>0</v>
       </c>
       <c r="C11">
-        <v>8.4125000000000005E-2</v>
+        <v>2.6315999999999999E-2</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>9.4979999999999995E-3</v>
+        <v>0</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -1029,13 +1029,13 @@
         <v>0</v>
       </c>
       <c r="K11">
-        <v>0.654003</v>
+        <v>0.78947400000000001</v>
       </c>
       <c r="L11">
         <v>0</v>
       </c>
       <c r="M11">
-        <v>0.19403000000000001</v>
+        <v>0.16447400000000001</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -1047,7 +1047,7 @@
         <v>0</v>
       </c>
       <c r="Q11">
-        <v>1.3569999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="R11">
         <v>0</v>
@@ -1059,63 +1059,63 @@
         <v>0</v>
       </c>
       <c r="U11">
-        <v>5.6987999999999997E-2</v>
+        <v>1.9737000000000001E-2</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A12">
-        <v>2.075E-3</v>
+        <v>1.157E-3</v>
       </c>
       <c r="B12">
-        <v>4.4099999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="C12">
-        <v>2.3349999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="D12">
-        <v>2.1530000000000001E-2</v>
+        <v>8.1019999999999998E-3</v>
       </c>
       <c r="E12">
-        <v>5.1900000000000004E-4</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>8.8199999999999997E-3</v>
+        <v>1.157E-3</v>
       </c>
       <c r="G12">
         <v>0</v>
       </c>
       <c r="H12">
-        <v>2.5900000000000001E-4</v>
+        <v>0</v>
       </c>
       <c r="I12">
-        <v>5.1900000000000004E-4</v>
+        <v>0</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
-        <v>1.5560000000000001E-3</v>
+        <v>2.3149999999999998E-3</v>
       </c>
       <c r="L12">
-        <v>0.81789900000000004</v>
+        <v>0.89583299999999999</v>
       </c>
       <c r="M12">
-        <v>2.5900000000000001E-4</v>
+        <v>0</v>
       </c>
       <c r="N12">
-        <v>0.114916</v>
+        <v>8.3333000000000004E-2</v>
       </c>
       <c r="O12">
-        <v>3.372E-3</v>
+        <v>1.157E-3</v>
       </c>
       <c r="P12">
-        <v>1.0380000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="Q12">
-        <v>2.5900000000000001E-4</v>
+        <v>0</v>
       </c>
       <c r="R12">
-        <v>5.1900000000000004E-4</v>
+        <v>0</v>
       </c>
       <c r="S12">
         <v>0</v>
@@ -1124,7 +1124,7 @@
         <v>0</v>
       </c>
       <c r="U12">
-        <v>1.9715E-2</v>
+        <v>6.9439999999999997E-3</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.45">
@@ -1132,16 +1132,16 @@
         <v>0</v>
       </c>
       <c r="B13">
-        <v>1.908E-3</v>
+        <v>0</v>
       </c>
       <c r="C13">
-        <v>3.2443E-2</v>
+        <v>0</v>
       </c>
       <c r="D13">
         <v>0</v>
       </c>
       <c r="E13">
-        <v>3.4351E-2</v>
+        <v>0</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -1159,16 +1159,16 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <v>6.2977000000000005E-2</v>
+        <v>8.1081E-2</v>
       </c>
       <c r="L13">
         <v>0</v>
       </c>
       <c r="M13">
-        <v>0.70801499999999995</v>
+        <v>0.81081099999999995</v>
       </c>
       <c r="N13">
-        <v>1.908E-3</v>
+        <v>0</v>
       </c>
       <c r="O13">
         <v>0</v>
@@ -1177,7 +1177,7 @@
         <v>0</v>
       </c>
       <c r="Q13">
-        <v>1.908E-3</v>
+        <v>0</v>
       </c>
       <c r="R13">
         <v>0</v>
@@ -1189,7 +1189,7 @@
         <v>0</v>
       </c>
       <c r="U13">
-        <v>0.15648899999999999</v>
+        <v>0.108108</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.45">
@@ -1197,25 +1197,25 @@
         <v>0</v>
       </c>
       <c r="B14">
-        <v>4.3909999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="C14">
-        <v>2.1949999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="D14">
-        <v>1.3172E-2</v>
+        <v>9.5239999999999995E-3</v>
       </c>
       <c r="E14">
-        <v>1.098E-3</v>
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>3.7322000000000001E-2</v>
+        <v>1.9047999999999999E-2</v>
       </c>
       <c r="G14">
         <v>0</v>
       </c>
       <c r="H14">
-        <v>1.098E-3</v>
+        <v>0</v>
       </c>
       <c r="I14">
         <v>0</v>
@@ -1224,28 +1224,28 @@
         <v>0</v>
       </c>
       <c r="K14">
-        <v>1.098E-3</v>
+        <v>0</v>
       </c>
       <c r="L14">
-        <v>0.12842999999999999</v>
+        <v>0.15238099999999999</v>
       </c>
       <c r="M14">
-        <v>4.3909999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="N14">
-        <v>0.61909999999999998</v>
+        <v>0.72380999999999995</v>
       </c>
       <c r="O14">
-        <v>6.5859999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="P14">
-        <v>1.098E-3</v>
+        <v>0</v>
       </c>
       <c r="Q14">
-        <v>1.0977000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="R14">
-        <v>1.098E-3</v>
+        <v>0</v>
       </c>
       <c r="S14">
         <v>0</v>
@@ -1254,7 +1254,7 @@
         <v>0</v>
       </c>
       <c r="U14">
-        <v>0.16794700000000001</v>
+        <v>9.5238000000000003E-2</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.45">
@@ -1265,19 +1265,19 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>2.5773000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="D15">
         <v>0</v>
       </c>
       <c r="E15">
-        <v>5.1549999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="F15">
         <v>0</v>
       </c>
       <c r="G15">
-        <v>2.5773000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -1292,22 +1292,22 @@
         <v>0</v>
       </c>
       <c r="L15">
-        <v>5.1549999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="M15">
-        <v>5.1549999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="N15">
-        <v>5.1549999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="O15">
-        <v>0.59793799999999997</v>
+        <v>0.76190500000000005</v>
       </c>
       <c r="P15">
         <v>0</v>
       </c>
       <c r="Q15">
-        <v>0.22164900000000001</v>
+        <v>0.14285700000000001</v>
       </c>
       <c r="R15">
         <v>0</v>
@@ -1319,7 +1319,7 @@
         <v>0</v>
       </c>
       <c r="U15">
-        <v>0.108247</v>
+        <v>9.5238000000000003E-2</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.45">
@@ -1333,13 +1333,13 @@
         <v>0</v>
       </c>
       <c r="D16">
-        <v>4.1667000000000003E-2</v>
+        <v>0</v>
       </c>
       <c r="E16">
         <v>0</v>
       </c>
       <c r="F16">
-        <v>3.4722000000000003E-2</v>
+        <v>0</v>
       </c>
       <c r="G16">
         <v>0</v>
@@ -1348,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="I16">
-        <v>6.9439999999999997E-3</v>
+        <v>0</v>
       </c>
       <c r="J16">
         <v>0</v>
@@ -1357,25 +1357,25 @@
         <v>0</v>
       </c>
       <c r="L16">
-        <v>1.3889E-2</v>
+        <v>0</v>
       </c>
       <c r="M16">
         <v>0</v>
       </c>
       <c r="N16">
-        <v>1.3889E-2</v>
+        <v>0</v>
       </c>
       <c r="O16">
-        <v>2.0833000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="P16">
-        <v>0.36805599999999999</v>
+        <v>0.63636400000000004</v>
       </c>
       <c r="Q16">
         <v>0</v>
       </c>
       <c r="R16">
-        <v>1.3889E-2</v>
+        <v>0</v>
       </c>
       <c r="S16">
         <v>0</v>
@@ -1384,7 +1384,7 @@
         <v>0</v>
       </c>
       <c r="U16">
-        <v>0.48611100000000002</v>
+        <v>0.36363600000000001</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.45">
@@ -1395,19 +1395,19 @@
         <v>0</v>
       </c>
       <c r="C17">
-        <v>1.5625E-2</v>
+        <v>0</v>
       </c>
       <c r="D17">
         <v>0</v>
       </c>
       <c r="E17">
-        <v>3.125E-2</v>
+        <v>0</v>
       </c>
       <c r="F17">
-        <v>1.5625E-2</v>
+        <v>0</v>
       </c>
       <c r="G17">
-        <v>1.5625E-2</v>
+        <v>0</v>
       </c>
       <c r="H17">
         <v>0</v>
@@ -1428,16 +1428,16 @@
         <v>0</v>
       </c>
       <c r="N17">
-        <v>1.5625E-2</v>
+        <v>0</v>
       </c>
       <c r="O17">
-        <v>3.125E-2</v>
+        <v>0</v>
       </c>
       <c r="P17">
         <v>0</v>
       </c>
       <c r="Q17">
-        <v>0.5625</v>
+        <v>0</v>
       </c>
       <c r="R17">
         <v>0</v>
@@ -1449,7 +1449,7 @@
         <v>0</v>
       </c>
       <c r="U17">
-        <v>0.3125</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.45">
@@ -1505,16 +1505,16 @@
         <v>0</v>
       </c>
       <c r="R18">
-        <v>0.72727299999999995</v>
+        <v>0</v>
       </c>
       <c r="S18">
         <v>0</v>
       </c>
       <c r="T18">
-        <v>9.0909000000000004E-2</v>
+        <v>0</v>
       </c>
       <c r="U18">
-        <v>0.18181800000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.45">
@@ -1573,13 +1573,13 @@
         <v>0</v>
       </c>
       <c r="S19">
-        <v>0.83333299999999999</v>
+        <v>0</v>
       </c>
       <c r="T19">
         <v>0</v>
       </c>
       <c r="U19">
-        <v>0.16666700000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.45">
@@ -1644,7 +1644,7 @@
         <v>0</v>
       </c>
       <c r="U20">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add other thstack codes
</commit_message>
<xml_diff>
--- a/Belle2/data.xlsx
+++ b/Belle2/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\purol\OneDrive\바탕 화면\github\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28BC4EEA-4389-4518-94E8-57B845B649E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D1F2FAF-4072-4C0A-B3F0-8FDC4996EC26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -349,22 +349,22 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A1">
-        <v>0.73900999999999994</v>
+        <v>0.80368099999999998</v>
       </c>
       <c r="B1">
-        <v>0.19405900000000001</v>
+        <v>0.157975</v>
       </c>
       <c r="C1">
-        <v>4.3559999999999996E-3</v>
+        <v>7.6689999999999996E-3</v>
       </c>
       <c r="D1">
-        <v>2.3760000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="E1">
         <v>0</v>
       </c>
       <c r="F1">
-        <v>1.5839999999999999E-3</v>
+        <v>7.67E-4</v>
       </c>
       <c r="G1">
         <v>0</v>
@@ -379,16 +379,16 @@
         <v>0</v>
       </c>
       <c r="K1">
-        <v>3.9599999999999998E-4</v>
+        <v>0</v>
       </c>
       <c r="L1">
-        <v>3.2079000000000003E-2</v>
+        <v>1.1502999999999999E-2</v>
       </c>
       <c r="M1">
         <v>0</v>
       </c>
       <c r="N1">
-        <v>5.1489999999999999E-3</v>
+        <v>2.3010000000000001E-3</v>
       </c>
       <c r="O1">
         <v>0</v>
@@ -409,27 +409,27 @@
         <v>0</v>
       </c>
       <c r="U1">
-        <v>2.0990000000000002E-2</v>
+        <v>1.6104E-2</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A2">
-        <v>5.1382999999999998E-2</v>
+        <v>6.8825999999999998E-2</v>
       </c>
       <c r="B2">
-        <v>0.79130400000000001</v>
+        <v>0.85829999999999995</v>
       </c>
       <c r="C2">
-        <v>8.6960000000000006E-3</v>
+        <v>2.0243000000000001E-2</v>
       </c>
       <c r="D2">
-        <v>3.9529999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>1.5809999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <v>4.7429999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -441,22 +441,22 @@
         <v>0</v>
       </c>
       <c r="J2">
-        <v>7.9100000000000004E-4</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>0</v>
       </c>
       <c r="L2">
-        <v>1.1067E-2</v>
+        <v>0</v>
       </c>
       <c r="M2">
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1.8971999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <v>7.9100000000000004E-4</v>
+        <v>0</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -474,7 +474,7 @@
         <v>0</v>
       </c>
       <c r="U2">
-        <v>0.10671899999999999</v>
+        <v>5.2631999999999998E-2</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.45">
@@ -485,13 +485,13 @@
         <v>0</v>
       </c>
       <c r="C3">
-        <v>0.83759399999999995</v>
+        <v>0.91025599999999995</v>
       </c>
       <c r="D3">
-        <v>1.5039999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>0.12781999999999999</v>
+        <v>7.2650000000000006E-2</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -509,25 +509,25 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>3.0079999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="L3">
-        <v>4.5110000000000003E-3</v>
+        <v>0</v>
       </c>
       <c r="M3">
-        <v>1.5039999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="N3">
         <v>0</v>
       </c>
       <c r="O3">
-        <v>1.2030000000000001E-2</v>
+        <v>4.274E-3</v>
       </c>
       <c r="P3">
         <v>0</v>
       </c>
       <c r="Q3">
-        <v>1.5039999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="R3">
         <v>0</v>
@@ -539,7 +539,7 @@
         <v>0</v>
       </c>
       <c r="U3">
-        <v>1.0526000000000001E-2</v>
+        <v>1.2821000000000001E-2</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.45">
@@ -547,28 +547,28 @@
         <v>0</v>
       </c>
       <c r="B4">
-        <v>3.509E-3</v>
+        <v>0</v>
       </c>
       <c r="C4">
-        <v>1.4035000000000001E-2</v>
+        <v>2.3973000000000001E-2</v>
       </c>
       <c r="D4">
-        <v>0.64736800000000005</v>
+        <v>0.71917799999999998</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0.221053</v>
+        <v>0.188356</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>3.4250000000000001E-3</v>
       </c>
       <c r="H4">
-        <v>1.7539999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>1.7539999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -577,22 +577,22 @@
         <v>0</v>
       </c>
       <c r="L4">
-        <v>2.4560999999999999E-2</v>
+        <v>6.8490000000000001E-3</v>
       </c>
       <c r="M4">
         <v>0</v>
       </c>
       <c r="N4">
-        <v>5.2630000000000003E-3</v>
+        <v>3.4250000000000001E-3</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>1.2281E-2</v>
+        <v>1.7122999999999999E-2</v>
       </c>
       <c r="Q4">
-        <v>1.7539999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="R4">
         <v>0</v>
@@ -604,7 +604,7 @@
         <v>0</v>
       </c>
       <c r="U4">
-        <v>6.6667000000000004E-2</v>
+        <v>3.7671000000000003E-2</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.45">
@@ -615,19 +615,19 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>0.20547899999999999</v>
+        <v>0.14285700000000001</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>0.58219200000000004</v>
+        <v>0.71428599999999998</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
-        <v>1.3698999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -642,22 +642,22 @@
         <v>0</v>
       </c>
       <c r="L5">
-        <v>6.8490000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="M5">
-        <v>2.0548E-2</v>
+        <v>0</v>
       </c>
       <c r="N5">
         <v>0</v>
       </c>
       <c r="O5">
-        <v>2.0548E-2</v>
+        <v>0</v>
       </c>
       <c r="P5">
         <v>0</v>
       </c>
       <c r="Q5">
-        <v>2.0548E-2</v>
+        <v>0</v>
       </c>
       <c r="R5">
         <v>0</v>
@@ -669,7 +669,7 @@
         <v>0</v>
       </c>
       <c r="U5">
-        <v>0.130137</v>
+        <v>0.14285700000000001</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.45">
@@ -677,19 +677,19 @@
         <v>0</v>
       </c>
       <c r="B6">
-        <v>7.2459999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6">
-        <v>8.6957000000000007E-2</v>
+        <v>0.18181800000000001</v>
       </c>
       <c r="E6">
-        <v>7.2459999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="F6">
-        <v>0.65942000000000001</v>
+        <v>0.77272700000000005</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -707,19 +707,19 @@
         <v>0</v>
       </c>
       <c r="L6">
-        <v>7.2459999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="M6">
         <v>0</v>
       </c>
       <c r="N6">
-        <v>5.7971000000000002E-2</v>
+        <v>0</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>7.2459999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -734,7 +734,7 @@
         <v>0</v>
       </c>
       <c r="U6">
-        <v>0.16666700000000001</v>
+        <v>4.5455000000000002E-2</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.45">
@@ -757,7 +757,7 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>0.33333299999999999</v>
+        <v>1</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -781,13 +781,13 @@
         <v>0</v>
       </c>
       <c r="O7">
-        <v>6.6667000000000004E-2</v>
+        <v>0</v>
       </c>
       <c r="P7">
         <v>0</v>
       </c>
       <c r="Q7">
-        <v>6.6667000000000004E-2</v>
+        <v>0</v>
       </c>
       <c r="R7">
         <v>0</v>
@@ -799,7 +799,7 @@
         <v>0</v>
       </c>
       <c r="U7">
-        <v>0.53333299999999995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.45">
@@ -813,7 +813,7 @@
         <v>0</v>
       </c>
       <c r="D8">
-        <v>4.8779999999999997E-2</v>
+        <v>0</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -825,13 +825,13 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>0.82926800000000001</v>
+        <v>0.92857100000000004</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8">
-        <v>0.121951</v>
+        <v>7.1429000000000006E-2</v>
       </c>
       <c r="K8">
         <v>0</v>
@@ -961,7 +961,7 @@
         <v>0</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -1005,13 +1005,13 @@
         <v>0</v>
       </c>
       <c r="C11">
-        <v>8.1559999999999994E-2</v>
+        <v>0</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>1.0638E-2</v>
+        <v>0</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -1029,13 +1029,13 @@
         <v>0</v>
       </c>
       <c r="K11">
-        <v>0.62766</v>
+        <v>0.80821900000000002</v>
       </c>
       <c r="L11">
         <v>0</v>
       </c>
       <c r="M11">
-        <v>0.25531900000000002</v>
+        <v>0.164384</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -1059,7 +1059,7 @@
         <v>0</v>
       </c>
       <c r="U11">
-        <v>2.4823000000000001E-2</v>
+        <v>2.7397000000000001E-2</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.45">
@@ -1067,19 +1067,19 @@
         <v>0</v>
       </c>
       <c r="B12">
-        <v>2.0630000000000002E-3</v>
+        <v>0</v>
       </c>
       <c r="C12">
-        <v>1.3760000000000001E-3</v>
+        <v>1.1919999999999999E-3</v>
       </c>
       <c r="D12">
-        <v>1.7881999999999999E-2</v>
+        <v>5.9589999999999999E-3</v>
       </c>
       <c r="E12">
-        <v>6.8800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>1.238E-2</v>
+        <v>0</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -1094,19 +1094,19 @@
         <v>0</v>
       </c>
       <c r="K12">
-        <v>1.3760000000000001E-3</v>
+        <v>2.3839999999999998E-3</v>
       </c>
       <c r="L12">
-        <v>0.842503</v>
+        <v>0.91656700000000002</v>
       </c>
       <c r="M12">
-        <v>1.3760000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="N12">
-        <v>0.101788</v>
+        <v>6.1978999999999999E-2</v>
       </c>
       <c r="O12">
-        <v>2.751E-3</v>
+        <v>1.1919999999999999E-3</v>
       </c>
       <c r="P12">
         <v>0</v>
@@ -1124,7 +1124,7 @@
         <v>0</v>
       </c>
       <c r="U12">
-        <v>1.5817999999999999E-2</v>
+        <v>1.0727E-2</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.45">
@@ -1135,13 +1135,13 @@
         <v>0</v>
       </c>
       <c r="C13">
-        <v>3.8674E-2</v>
+        <v>0</v>
       </c>
       <c r="D13">
         <v>0</v>
       </c>
       <c r="E13">
-        <v>4.4199000000000002E-2</v>
+        <v>0</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -1159,19 +1159,19 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <v>6.0773000000000001E-2</v>
+        <v>6.4516000000000004E-2</v>
       </c>
       <c r="L13">
         <v>0</v>
       </c>
       <c r="M13">
-        <v>0.74033099999999996</v>
+        <v>0.80645199999999995</v>
       </c>
       <c r="N13">
         <v>0</v>
       </c>
       <c r="O13">
-        <v>5.5250000000000004E-3</v>
+        <v>0</v>
       </c>
       <c r="P13">
         <v>0</v>
@@ -1189,7 +1189,7 @@
         <v>0</v>
       </c>
       <c r="U13">
-        <v>0.110497</v>
+        <v>0.12903200000000001</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.45">
@@ -1197,19 +1197,19 @@
         <v>0</v>
       </c>
       <c r="B14">
-        <v>8.9549999999999994E-3</v>
+        <v>0</v>
       </c>
       <c r="C14">
-        <v>2.9849999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="D14">
-        <v>2.0896000000000001E-2</v>
+        <v>2.1739000000000001E-2</v>
       </c>
       <c r="E14">
-        <v>2.9849999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>3.2835999999999997E-2</v>
+        <v>0</v>
       </c>
       <c r="G14">
         <v>0</v>
@@ -1224,19 +1224,19 @@
         <v>0</v>
       </c>
       <c r="K14">
-        <v>2.9849999999999998E-3</v>
+        <v>0</v>
       </c>
       <c r="L14">
-        <v>0.14029900000000001</v>
+        <v>0.23913000000000001</v>
       </c>
       <c r="M14">
-        <v>5.9699999999999996E-3</v>
+        <v>0</v>
       </c>
       <c r="N14">
-        <v>0.66268700000000003</v>
+        <v>0.69565200000000005</v>
       </c>
       <c r="O14">
-        <v>2.9849999999999998E-3</v>
+        <v>1.0869999999999999E-2</v>
       </c>
       <c r="P14">
         <v>0</v>
@@ -1254,7 +1254,7 @@
         <v>0</v>
       </c>
       <c r="U14">
-        <v>0.11641799999999999</v>
+        <v>3.2608999999999999E-2</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.45">
@@ -1265,7 +1265,7 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>1.5152000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -1292,22 +1292,22 @@
         <v>0</v>
       </c>
       <c r="L15">
-        <v>1.5152000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="M15">
-        <v>1.5152000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="N15">
-        <v>1.5152000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="O15">
-        <v>0.5</v>
+        <v>0.80952400000000002</v>
       </c>
       <c r="P15">
-        <v>1.5152000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="Q15">
-        <v>0.34848499999999999</v>
+        <v>0.19047600000000001</v>
       </c>
       <c r="R15">
         <v>0</v>
@@ -1319,7 +1319,7 @@
         <v>0</v>
       </c>
       <c r="U15">
-        <v>7.5758000000000006E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.45">
@@ -1339,10 +1339,10 @@
         <v>0</v>
       </c>
       <c r="F16">
-        <v>2.3810000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>2.3810000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="H16">
         <v>0</v>
@@ -1363,13 +1363,13 @@
         <v>0</v>
       </c>
       <c r="N16">
-        <v>2.3810000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="O16">
         <v>0</v>
       </c>
       <c r="P16">
-        <v>0.33333299999999999</v>
+        <v>0.40909099999999998</v>
       </c>
       <c r="Q16">
         <v>0</v>
@@ -1384,7 +1384,7 @@
         <v>0</v>
       </c>
       <c r="U16">
-        <v>0.59523800000000004</v>
+        <v>0.59090900000000002</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.45">
@@ -1407,7 +1407,7 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>7.6923000000000005E-2</v>
+        <v>0</v>
       </c>
       <c r="H17">
         <v>0</v>
@@ -1431,13 +1431,13 @@
         <v>0</v>
       </c>
       <c r="O17">
-        <v>0.15384600000000001</v>
+        <v>0</v>
       </c>
       <c r="P17">
         <v>0</v>
       </c>
       <c r="Q17">
-        <v>0.538462</v>
+        <v>0</v>
       </c>
       <c r="R17">
         <v>0</v>
@@ -1449,7 +1449,7 @@
         <v>0</v>
       </c>
       <c r="U17">
-        <v>0.230769</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.45">
@@ -1573,7 +1573,7 @@
         <v>0</v>
       </c>
       <c r="S19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T19">
         <v>0</v>

</xml_diff>

<commit_message>
max digit for THSTACK plot
</commit_message>
<xml_diff>
--- a/Belle2/data.xlsx
+++ b/Belle2/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25225"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\purol\OneDrive\바탕 화면\github\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13ED01AC-3C2C-43F5-AC4A-DCD4871F5B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5C13EA2-8994-4223-97B1-B3AD0F2A7ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -349,25 +349,25 @@
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.45">
       <c r="A1">
-        <v>0.55093199999999998</v>
+        <v>0.52534400000000003</v>
       </c>
       <c r="B1">
-        <v>0.33899899999999999</v>
+        <v>0.35337000000000002</v>
       </c>
       <c r="C1">
-        <v>1.6254999999999999E-2</v>
+        <v>1.7548999999999999E-2</v>
       </c>
       <c r="D1">
-        <v>2.8930000000000002E-3</v>
+        <v>3.1250000000000002E-3</v>
       </c>
       <c r="E1">
-        <v>1.946E-3</v>
+        <v>2.3549999999999999E-3</v>
       </c>
       <c r="F1">
-        <v>2.183E-3</v>
+        <v>2.4250000000000001E-3</v>
       </c>
       <c r="G1">
-        <v>2.5999999999999998E-5</v>
+        <v>4.6999999999999997E-5</v>
       </c>
       <c r="H1">
         <v>0</v>
@@ -376,90 +376,90 @@
         <v>0</v>
       </c>
       <c r="J1">
-        <v>1.2676E-2</v>
+        <v>1.4482999999999999E-2</v>
       </c>
       <c r="K1">
-        <v>5.3000000000000001E-5</v>
+        <v>6.9999999999999994E-5</v>
       </c>
       <c r="L1">
-        <v>1.3100000000000001E-4</v>
+        <v>1.63E-4</v>
       </c>
       <c r="M1">
-        <v>2.1000000000000001E-4</v>
+        <v>2.33E-4</v>
       </c>
       <c r="N1">
-        <v>7.8999999999999996E-5</v>
+        <v>9.2999999999999997E-5</v>
       </c>
       <c r="O1">
         <v>0</v>
       </c>
       <c r="P1">
-        <v>1.5200000000000001E-4</v>
+        <v>1.35E-4</v>
       </c>
       <c r="Q1">
-        <v>3.6083999999999998E-2</v>
+        <v>3.7516000000000001E-2</v>
       </c>
       <c r="R1">
-        <v>2.6999999999999999E-5</v>
+        <v>9.1000000000000003E-5</v>
       </c>
       <c r="S1">
-        <v>4.7219999999999996E-3</v>
+        <v>5.2919999999999998E-3</v>
       </c>
       <c r="T1">
-        <v>1.5899999999999999E-4</v>
+        <v>2.3499999999999999E-4</v>
       </c>
       <c r="U1">
-        <v>0</v>
+        <v>2.4000000000000001E-5</v>
       </c>
       <c r="V1">
-        <v>2.6999999999999999E-5</v>
+        <v>2.4000000000000001E-5</v>
       </c>
       <c r="W1">
-        <v>5.3000000000000001E-5</v>
+        <v>4.6999999999999997E-5</v>
       </c>
       <c r="X1">
         <v>0</v>
       </c>
       <c r="Y1">
-        <v>2.6999999999999999E-5</v>
+        <v>2.4000000000000001E-5</v>
       </c>
       <c r="Z1">
-        <v>1.8599999999999999E-4</v>
+        <v>2.5900000000000001E-4</v>
       </c>
       <c r="AA1">
         <v>0</v>
       </c>
       <c r="AB1">
-        <v>0</v>
+        <v>2.4000000000000001E-5</v>
       </c>
       <c r="AC1">
         <v>0</v>
       </c>
       <c r="AD1">
-        <v>0</v>
+        <v>4.6999999999999997E-5</v>
       </c>
       <c r="AE1">
-        <v>3.2181000000000001E-2</v>
+        <v>3.7026000000000003E-2</v>
       </c>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.45">
       <c r="A2">
-        <v>1.7243999999999999E-2</v>
+        <v>1.9060000000000001E-2</v>
       </c>
       <c r="B2">
-        <v>0.84068799999999999</v>
+        <v>0.82382299999999997</v>
       </c>
       <c r="C2">
-        <v>9.7090000000000006E-3</v>
+        <v>8.8350000000000008E-3</v>
       </c>
       <c r="D2">
-        <v>1.073E-3</v>
+        <v>2.2850000000000001E-3</v>
       </c>
       <c r="E2">
-        <v>4.7219999999999996E-3</v>
+        <v>5.1419999999999999E-3</v>
       </c>
       <c r="F2">
-        <v>2.3609999999999998E-3</v>
+        <v>1.523E-3</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -471,19 +471,19 @@
         <v>0</v>
       </c>
       <c r="J2">
-        <v>5.8599999999999999E-2</v>
+        <v>6.3413999999999998E-2</v>
       </c>
       <c r="K2">
-        <v>2.1499999999999999E-4</v>
+        <v>5.71E-4</v>
       </c>
       <c r="L2">
-        <v>2.1499999999999999E-4</v>
+        <v>1.9000000000000001E-4</v>
       </c>
       <c r="M2">
-        <v>2.1499999999999999E-4</v>
+        <v>1.9000000000000001E-4</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1.9000000000000001E-4</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -492,22 +492,22 @@
         <v>0</v>
       </c>
       <c r="Q2">
-        <v>6.0520000000000001E-3</v>
+        <v>6.1380000000000002E-3</v>
       </c>
       <c r="R2">
-        <v>1.0499999999999999E-3</v>
+        <v>1.8630000000000001E-3</v>
       </c>
       <c r="S2">
-        <v>1.1691E-2</v>
+        <v>1.2485E-2</v>
       </c>
       <c r="T2">
-        <v>2.1599999999999999E-4</v>
+        <v>1.92E-4</v>
       </c>
       <c r="U2">
         <v>0</v>
       </c>
       <c r="V2">
-        <v>2.1599999999999999E-4</v>
+        <v>1.92E-4</v>
       </c>
       <c r="W2">
         <v>0</v>
@@ -516,16 +516,16 @@
         <v>0</v>
       </c>
       <c r="Y2">
-        <v>2.1599999999999999E-4</v>
+        <v>1.92E-4</v>
       </c>
       <c r="Z2">
-        <v>6.4899999999999995E-4</v>
+        <v>5.7600000000000001E-4</v>
       </c>
       <c r="AA2">
         <v>0</v>
       </c>
       <c r="AB2">
-        <v>0</v>
+        <v>1.92E-4</v>
       </c>
       <c r="AC2">
         <v>0</v>
@@ -534,7 +534,7 @@
         <v>0</v>
       </c>
       <c r="AE2">
-        <v>4.4866000000000003E-2</v>
+        <v>5.2944999999999999E-2</v>
       </c>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.45">
@@ -545,31 +545,31 @@
         <v>0</v>
       </c>
       <c r="C3">
-        <v>0.881525</v>
+        <v>0.872201</v>
       </c>
       <c r="D3">
-        <v>2.4000000000000001E-4</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="E3">
-        <v>9.7247E-2</v>
+        <v>0.103076</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3">
-        <v>9.5799999999999998E-4</v>
+        <v>7.9900000000000001E-4</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>2.4000000000000001E-4</v>
+        <v>5.9900000000000003E-4</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>2.8739999999999998E-3</v>
+        <v>4.3949999999999996E-3</v>
       </c>
       <c r="L3">
         <v>0</v>
@@ -584,25 +584,25 @@
         <v>0</v>
       </c>
       <c r="P3">
-        <v>2.7659999999999998E-3</v>
+        <v>2.5379999999999999E-3</v>
       </c>
       <c r="Q3">
-        <v>7.2499999999999995E-4</v>
+        <v>6.0400000000000004E-4</v>
       </c>
       <c r="R3">
-        <v>3.068E-3</v>
+        <v>3.3349999999999999E-3</v>
       </c>
       <c r="S3">
-        <v>2.42E-4</v>
+        <v>2.0100000000000001E-4</v>
       </c>
       <c r="T3">
-        <v>4.5900000000000003E-3</v>
+        <v>4.8349999999999999E-3</v>
       </c>
       <c r="U3">
         <v>0</v>
       </c>
       <c r="V3">
-        <v>1.2080000000000001E-3</v>
+        <v>1.8129999999999999E-3</v>
       </c>
       <c r="W3">
         <v>0</v>
@@ -611,13 +611,13 @@
         <v>0</v>
       </c>
       <c r="Y3">
-        <v>0</v>
+        <v>2.0100000000000001E-4</v>
       </c>
       <c r="Z3">
         <v>0</v>
       </c>
       <c r="AA3">
-        <v>2.42E-4</v>
+        <v>4.0299999999999998E-4</v>
       </c>
       <c r="AB3">
         <v>0</v>
@@ -629,51 +629,51 @@
         <v>0</v>
       </c>
       <c r="AE3">
-        <v>4.0759999999999998E-3</v>
+        <v>4.7990000000000003E-3</v>
       </c>
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.45">
       <c r="A4">
-        <v>5.6800000000000004E-4</v>
+        <v>4.6200000000000001E-4</v>
       </c>
       <c r="B4">
-        <v>3.6939999999999998E-3</v>
+        <v>4.4089999999999997E-3</v>
       </c>
       <c r="C4">
-        <v>6.9560000000000004E-3</v>
+        <v>5.6569999999999997E-3</v>
       </c>
       <c r="D4">
-        <v>0.66210899999999995</v>
+        <v>0.64033899999999999</v>
       </c>
       <c r="E4">
-        <v>4.3199999999999998E-4</v>
+        <v>7.0200000000000004E-4</v>
       </c>
       <c r="F4">
-        <v>0.22919200000000001</v>
+        <v>0.23556299999999999</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>3.5100000000000002E-4</v>
       </c>
       <c r="H4">
-        <v>4.3199999999999998E-4</v>
+        <v>3.5100000000000002E-4</v>
       </c>
       <c r="I4">
-        <v>4.3199999999999998E-4</v>
+        <v>3.5100000000000002E-4</v>
       </c>
       <c r="J4">
-        <v>4.3199999999999998E-4</v>
+        <v>3.5100000000000002E-4</v>
       </c>
       <c r="K4">
         <v>0</v>
       </c>
       <c r="L4">
-        <v>1.7697000000000001E-2</v>
+        <v>2.3872000000000001E-2</v>
       </c>
       <c r="M4">
-        <v>4.3199999999999998E-4</v>
+        <v>7.0200000000000004E-4</v>
       </c>
       <c r="N4">
-        <v>4.3199999999999998E-4</v>
+        <v>3.5100000000000002E-4</v>
       </c>
       <c r="O4">
         <v>0</v>
@@ -682,25 +682,25 @@
         <v>0</v>
       </c>
       <c r="Q4">
-        <v>2.9062999999999999E-2</v>
+        <v>3.0456E-2</v>
       </c>
       <c r="R4">
         <v>0</v>
       </c>
       <c r="S4">
-        <v>1.1754000000000001E-2</v>
+        <v>1.3455E-2</v>
       </c>
       <c r="T4">
-        <v>4.35E-4</v>
+        <v>7.0799999999999997E-4</v>
       </c>
       <c r="U4">
-        <v>7.4009999999999996E-3</v>
+        <v>9.5600000000000008E-3</v>
       </c>
       <c r="V4">
-        <v>0</v>
+        <v>3.5399999999999999E-4</v>
       </c>
       <c r="W4">
-        <v>3.9179999999999996E-3</v>
+        <v>4.9569999999999996E-3</v>
       </c>
       <c r="X4">
         <v>0</v>
@@ -709,7 +709,7 @@
         <v>0</v>
       </c>
       <c r="Z4">
-        <v>4.35E-4</v>
+        <v>0</v>
       </c>
       <c r="AA4">
         <v>0</v>
@@ -724,7 +724,7 @@
         <v>0</v>
       </c>
       <c r="AE4">
-        <v>2.4188999999999999E-2</v>
+        <v>2.7047000000000002E-2</v>
       </c>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.45">
@@ -735,31 +735,31 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>0.181142</v>
+        <v>0.20831</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>0.64296900000000001</v>
+        <v>0.626946</v>
       </c>
       <c r="F5">
-        <v>3.215E-3</v>
+        <v>2.5799999999999998E-3</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>2.5799999999999998E-3</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
       <c r="I5">
-        <v>6.43E-3</v>
+        <v>2.5799999999999998E-3</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>6.1081999999999997E-2</v>
+        <v>6.7081000000000002E-2</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -777,22 +777,22 @@
         <v>0</v>
       </c>
       <c r="Q5">
-        <v>3.2420000000000001E-3</v>
+        <v>2.6020000000000001E-3</v>
       </c>
       <c r="R5">
-        <v>3.0972E-2</v>
+        <v>2.0041E-2</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>2.6020000000000001E-3</v>
       </c>
       <c r="T5">
-        <v>6.4850000000000003E-3</v>
+        <v>5.2040000000000003E-3</v>
       </c>
       <c r="U5">
         <v>0</v>
       </c>
       <c r="V5">
-        <v>1.2970000000000001E-2</v>
+        <v>1.0409E-2</v>
       </c>
       <c r="W5">
         <v>0</v>
@@ -801,13 +801,13 @@
         <v>0</v>
       </c>
       <c r="Y5">
-        <v>0</v>
+        <v>2.6020000000000001E-3</v>
       </c>
       <c r="Z5">
         <v>0</v>
       </c>
       <c r="AA5">
-        <v>6.4850000000000003E-3</v>
+        <v>2.6020000000000001E-3</v>
       </c>
       <c r="AB5">
         <v>0</v>
@@ -819,7 +819,7 @@
         <v>0</v>
       </c>
       <c r="AE5">
-        <v>4.5007999999999999E-2</v>
+        <v>4.3860000000000003E-2</v>
       </c>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.45">
@@ -827,19 +827,19 @@
         <v>0</v>
       </c>
       <c r="B6">
-        <v>5.8100000000000001E-3</v>
+        <v>2.5332E-2</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6">
-        <v>5.8104999999999997E-2</v>
+        <v>8.6379999999999998E-2</v>
       </c>
       <c r="E6">
-        <v>1.1620999999999999E-2</v>
+        <v>9.5980000000000006E-3</v>
       </c>
       <c r="F6">
-        <v>0.66239400000000004</v>
+        <v>0.60465899999999995</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -848,7 +848,7 @@
         <v>0</v>
       </c>
       <c r="I6">
-        <v>5.8100000000000001E-3</v>
+        <v>4.7990000000000003E-3</v>
       </c>
       <c r="J6">
         <v>0</v>
@@ -857,7 +857,7 @@
         <v>0</v>
       </c>
       <c r="L6">
-        <v>0.15107200000000001</v>
+        <v>0.13916799999999999</v>
       </c>
       <c r="M6">
         <v>0</v>
@@ -878,19 +878,19 @@
         <v>0</v>
       </c>
       <c r="S6">
-        <v>4.1022999999999997E-2</v>
+        <v>1.452E-2</v>
       </c>
       <c r="T6">
         <v>0</v>
       </c>
       <c r="U6">
-        <v>0</v>
+        <v>4.8399999999999997E-3</v>
       </c>
       <c r="V6">
         <v>0</v>
       </c>
       <c r="W6">
-        <v>1.1721000000000001E-2</v>
+        <v>1.452E-2</v>
       </c>
       <c r="X6">
         <v>0</v>
@@ -899,7 +899,7 @@
         <v>0</v>
       </c>
       <c r="Z6">
-        <v>5.8599999999999998E-3</v>
+        <v>9.6799999999999994E-3</v>
       </c>
       <c r="AA6">
         <v>0</v>
@@ -914,7 +914,7 @@
         <v>0</v>
       </c>
       <c r="AE6">
-        <v>4.6584E-2</v>
+        <v>8.6503999999999998E-2</v>
       </c>
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.45">
@@ -931,19 +931,19 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <v>4.1591999999999997E-2</v>
+        <v>3.3276E-2</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>3.3276E-2</v>
       </c>
       <c r="G7">
-        <v>0.37433</v>
+        <v>0.33276099999999997</v>
       </c>
       <c r="H7">
         <v>0</v>
       </c>
       <c r="I7">
-        <v>0.249553</v>
+        <v>0.26620899999999997</v>
       </c>
       <c r="J7">
         <v>0</v>
@@ -976,19 +976,19 @@
         <v>0</v>
       </c>
       <c r="T7">
-        <v>8.3899000000000001E-2</v>
+        <v>6.7124000000000003E-2</v>
       </c>
       <c r="U7">
         <v>0</v>
       </c>
       <c r="V7">
-        <v>4.1950000000000001E-2</v>
+        <v>6.7124000000000003E-2</v>
       </c>
       <c r="W7">
         <v>0</v>
       </c>
       <c r="X7">
-        <v>4.1950000000000001E-2</v>
+        <v>3.3562000000000002E-2</v>
       </c>
       <c r="Y7">
         <v>0</v>
@@ -1009,7 +1009,7 @@
         <v>0</v>
       </c>
       <c r="AE7">
-        <v>0.16672600000000001</v>
+        <v>0.16666700000000001</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.45">
@@ -1035,7 +1035,7 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>0.33333299999999999</v>
+        <v>0.2</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -1104,7 +1104,7 @@
         <v>0</v>
       </c>
       <c r="AE8">
-        <v>0.66666700000000001</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.45">
@@ -1133,7 +1133,7 @@
         <v>0</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -1204,22 +1204,22 @@
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.45">
       <c r="A10">
-        <v>1.1169999999999999E-2</v>
+        <v>9.1509999999999994E-3</v>
       </c>
       <c r="B10">
-        <v>0.311697</v>
+        <v>0.29202899999999998</v>
       </c>
       <c r="C10">
-        <v>5.2004000000000002E-2</v>
+        <v>5.2512999999999997E-2</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>2.3159999999999999E-3</v>
       </c>
       <c r="E10">
-        <v>1.6962999999999999E-2</v>
+        <v>1.6213000000000002E-2</v>
       </c>
       <c r="F10">
-        <v>8.482E-3</v>
+        <v>1.6213000000000002E-2</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -1231,13 +1231,13 @@
         <v>0</v>
       </c>
       <c r="J10">
-        <v>0.22334999999999999</v>
+        <v>0.22697999999999999</v>
       </c>
       <c r="K10">
-        <v>5.6540000000000002E-3</v>
+        <v>6.9480000000000002E-3</v>
       </c>
       <c r="L10">
-        <v>5.6540000000000002E-3</v>
+        <v>6.9480000000000002E-3</v>
       </c>
       <c r="M10">
         <v>0</v>
@@ -1252,13 +1252,13 @@
         <v>0</v>
       </c>
       <c r="Q10">
-        <v>2.8519999999999999E-3</v>
+        <v>8.9949999999999995E-3</v>
       </c>
       <c r="R10">
         <v>0</v>
       </c>
       <c r="S10">
-        <v>2.5663999999999999E-2</v>
+        <v>2.5696E-2</v>
       </c>
       <c r="T10">
         <v>0</v>
@@ -1279,10 +1279,10 @@
         <v>0</v>
       </c>
       <c r="Z10">
-        <v>5.7029999999999997E-3</v>
+        <v>9.3439999999999999E-3</v>
       </c>
       <c r="AA10">
-        <v>2.8519999999999999E-3</v>
+        <v>2.336E-3</v>
       </c>
       <c r="AB10">
         <v>0</v>
@@ -1294,7 +1294,7 @@
         <v>0</v>
       </c>
       <c r="AE10">
-        <v>0.327957</v>
+        <v>0.32431700000000002</v>
       </c>
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.45">
@@ -1311,7 +1311,7 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>0.41636800000000002</v>
+        <v>0.30769200000000002</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -1323,13 +1323,13 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>7.6923000000000005E-2</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11">
-        <v>0.166547</v>
+        <v>0.230769</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -1353,7 +1353,7 @@
         <v>0</v>
       </c>
       <c r="S11">
-        <v>8.3988999999999994E-2</v>
+        <v>0</v>
       </c>
       <c r="T11">
         <v>0</v>
@@ -1389,7 +1389,7 @@
         <v>0</v>
       </c>
       <c r="AE11">
-        <v>0.33309499999999997</v>
+        <v>0.38461499999999998</v>
       </c>
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.45">
@@ -1409,7 +1409,7 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>0.24946399999999999</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -1427,7 +1427,7 @@
         <v>0</v>
       </c>
       <c r="L12">
-        <v>0</v>
+        <v>0.24946399999999999</v>
       </c>
       <c r="M12">
         <v>0</v>
@@ -1448,7 +1448,7 @@
         <v>0</v>
       </c>
       <c r="S12">
-        <v>0</v>
+        <v>0.251608</v>
       </c>
       <c r="T12">
         <v>0</v>
@@ -1484,7 +1484,7 @@
         <v>0</v>
       </c>
       <c r="AE12">
-        <v>0</v>
+        <v>0.24946399999999999</v>
       </c>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.45">
@@ -1498,7 +1498,7 @@
         <v>0</v>
       </c>
       <c r="D13">
-        <v>1.081E-2</v>
+        <v>8.5100000000000002E-3</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -1525,13 +1525,13 @@
         <v>0</v>
       </c>
       <c r="M13">
-        <v>0.84860899999999995</v>
+        <v>0.80842199999999997</v>
       </c>
       <c r="N13">
         <v>0</v>
       </c>
       <c r="O13">
-        <v>0.113508</v>
+        <v>0.14466499999999999</v>
       </c>
       <c r="P13">
         <v>0</v>
@@ -1570,16 +1570,16 @@
         <v>0</v>
       </c>
       <c r="AB13">
-        <v>0</v>
+        <v>4.2909999999999997E-3</v>
       </c>
       <c r="AC13">
-        <v>5.4520000000000002E-3</v>
+        <v>8.5830000000000004E-3</v>
       </c>
       <c r="AD13">
         <v>0</v>
       </c>
       <c r="AE13">
-        <v>2.1621000000000001E-2</v>
+        <v>2.5529E-2</v>
       </c>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.45">
@@ -1715,13 +1715,13 @@
         <v>0</v>
       </c>
       <c r="M15">
-        <v>0.6</v>
+        <v>0.66666700000000001</v>
       </c>
       <c r="N15">
         <v>0</v>
       </c>
       <c r="O15">
-        <v>0.4</v>
+        <v>0.33333299999999999</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -1774,19 +1774,19 @@
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.45">
       <c r="A16">
-        <v>4.06E-4</v>
+        <v>3.3500000000000001E-4</v>
       </c>
       <c r="B16">
-        <v>1.01E-3</v>
+        <v>8.3500000000000002E-4</v>
       </c>
       <c r="C16">
-        <v>5.7501999999999998E-2</v>
+        <v>6.2019999999999999E-2</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <v>2.7720000000000002E-3</v>
+        <v>3.82E-3</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -1819,25 +1819,25 @@
         <v>0</v>
       </c>
       <c r="P16">
-        <v>0.57417899999999999</v>
+        <v>0.53519000000000005</v>
       </c>
       <c r="Q16">
-        <v>3.5430000000000001E-3</v>
+        <v>4.3930000000000002E-3</v>
       </c>
       <c r="R16">
-        <v>0.311282</v>
+        <v>0.334673</v>
       </c>
       <c r="S16">
-        <v>6.2100000000000002E-4</v>
+        <v>2.5700000000000001E-4</v>
       </c>
       <c r="T16">
-        <v>3.418E-3</v>
+        <v>3.852E-3</v>
       </c>
       <c r="U16">
         <v>0</v>
       </c>
       <c r="V16">
-        <v>1.554E-3</v>
+        <v>1.284E-3</v>
       </c>
       <c r="W16">
         <v>0</v>
@@ -1846,16 +1846,16 @@
         <v>0</v>
       </c>
       <c r="Y16">
-        <v>1.0874999999999999E-2</v>
+        <v>1.3355000000000001E-2</v>
       </c>
       <c r="Z16">
-        <v>0</v>
+        <v>2.5700000000000001E-4</v>
       </c>
       <c r="AA16">
         <v>0</v>
       </c>
       <c r="AB16">
-        <v>3.1100000000000002E-4</v>
+        <v>2.5700000000000001E-4</v>
       </c>
       <c r="AC16">
         <v>0</v>
@@ -1864,27 +1864,27 @@
         <v>0</v>
       </c>
       <c r="AE16">
-        <v>3.2528000000000001E-2</v>
+        <v>3.9472E-2</v>
       </c>
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.45">
       <c r="A17">
-        <v>1.369E-3</v>
+        <v>1.5590000000000001E-3</v>
       </c>
       <c r="B17">
-        <v>1.1509999999999999E-3</v>
+        <v>1.8370000000000001E-3</v>
       </c>
       <c r="C17">
-        <v>5.1999999999999995E-4</v>
+        <v>7.6000000000000004E-4</v>
       </c>
       <c r="D17">
-        <v>8.4919999999999995E-3</v>
+        <v>9.8390000000000005E-3</v>
       </c>
       <c r="E17">
-        <v>2.5999999999999998E-4</v>
+        <v>2.22E-4</v>
       </c>
       <c r="F17">
-        <v>1.82E-3</v>
+        <v>2.5149999999999999E-3</v>
       </c>
       <c r="G17">
         <v>0</v>
@@ -1893,19 +1893,19 @@
         <v>0</v>
       </c>
       <c r="I17">
-        <v>8.7000000000000001E-5</v>
+        <v>7.3999999999999996E-5</v>
       </c>
       <c r="J17">
-        <v>2.5999999999999998E-4</v>
+        <v>2.22E-4</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
       <c r="L17">
-        <v>8.7000000000000001E-5</v>
+        <v>7.3999999999999996E-5</v>
       </c>
       <c r="M17">
-        <v>8.7000000000000001E-5</v>
+        <v>7.3999999999999996E-5</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -1914,28 +1914,28 @@
         <v>0</v>
       </c>
       <c r="P17">
-        <v>0</v>
+        <v>2.5599999999999999E-4</v>
       </c>
       <c r="Q17">
-        <v>0.87557399999999996</v>
+        <v>0.85677000000000003</v>
       </c>
       <c r="R17">
-        <v>8.7000000000000001E-5</v>
+        <v>7.4999999999999993E-5</v>
       </c>
       <c r="S17">
-        <v>9.6925999999999998E-2</v>
+        <v>0.109162</v>
       </c>
       <c r="T17">
-        <v>2.5349999999999999E-3</v>
+        <v>2.9849999999999998E-3</v>
       </c>
       <c r="U17">
-        <v>7.8700000000000005E-4</v>
+        <v>6.7199999999999996E-4</v>
       </c>
       <c r="V17">
-        <v>1.75E-4</v>
+        <v>3.7300000000000001E-4</v>
       </c>
       <c r="W17">
-        <v>5.2400000000000005E-4</v>
+        <v>5.22E-4</v>
       </c>
       <c r="X17">
         <v>0</v>
@@ -1944,7 +1944,7 @@
         <v>0</v>
       </c>
       <c r="Z17">
-        <v>4.6319999999999998E-3</v>
+        <v>6.1180000000000002E-3</v>
       </c>
       <c r="AA17">
         <v>0</v>
@@ -1953,13 +1953,13 @@
         <v>0</v>
       </c>
       <c r="AC17">
-        <v>8.7000000000000001E-5</v>
+        <v>7.4999999999999993E-5</v>
       </c>
       <c r="AD17">
-        <v>0</v>
+        <v>7.4999999999999993E-5</v>
       </c>
       <c r="AE17">
-        <v>4.5409999999999999E-3</v>
+        <v>5.7400000000000003E-3</v>
       </c>
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.45">
@@ -1967,16 +1967,16 @@
         <v>0</v>
       </c>
       <c r="B18">
-        <v>1.2459999999999999E-3</v>
+        <v>1.127E-3</v>
       </c>
       <c r="C18">
-        <v>1.3501000000000001E-2</v>
+        <v>1.4147E-2</v>
       </c>
       <c r="D18">
         <v>0</v>
       </c>
       <c r="E18">
-        <v>1.7443E-2</v>
+        <v>2.2532E-2</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -1994,7 +1994,7 @@
         <v>0</v>
       </c>
       <c r="K18">
-        <v>0</v>
+        <v>1.127E-3</v>
       </c>
       <c r="L18">
         <v>0</v>
@@ -2009,25 +2009,25 @@
         <v>0</v>
       </c>
       <c r="P18">
-        <v>2.5898999999999998E-2</v>
+        <v>2.4719000000000001E-2</v>
       </c>
       <c r="Q18">
-        <v>0</v>
+        <v>3.2390000000000001E-3</v>
       </c>
       <c r="R18">
-        <v>0.838866</v>
+        <v>0.81493700000000002</v>
       </c>
       <c r="S18">
         <v>0</v>
       </c>
       <c r="T18">
-        <v>1.2570000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="U18">
         <v>0</v>
       </c>
       <c r="V18">
-        <v>1.2570000000000001E-3</v>
+        <v>3.4090000000000001E-3</v>
       </c>
       <c r="W18">
         <v>0</v>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="Y18">
-        <v>4.3982E-2</v>
+        <v>5.2268000000000002E-2</v>
       </c>
       <c r="Z18">
-        <v>1.2570000000000001E-3</v>
+        <v>1.1360000000000001E-3</v>
       </c>
       <c r="AA18">
         <v>0</v>
@@ -2054,7 +2054,7 @@
         <v>0</v>
       </c>
       <c r="AE18">
-        <v>5.5292000000000001E-2</v>
+        <v>6.1358999999999997E-2</v>
       </c>
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.45">
@@ -2062,19 +2062,19 @@
         <v>0</v>
       </c>
       <c r="B19">
-        <v>7.0939999999999996E-3</v>
+        <v>9.1249999999999994E-3</v>
       </c>
       <c r="C19">
         <v>0</v>
       </c>
       <c r="D19">
-        <v>1.2428E-2</v>
+        <v>1.3365999999999999E-2</v>
       </c>
       <c r="E19">
         <v>0</v>
       </c>
       <c r="F19">
-        <v>1.6948000000000001E-2</v>
+        <v>3.1505999999999999E-2</v>
       </c>
       <c r="G19">
         <v>0</v>
@@ -2086,16 +2086,16 @@
         <v>0</v>
       </c>
       <c r="J19">
-        <v>2.2599999999999999E-3</v>
+        <v>2.8639999999999998E-3</v>
       </c>
       <c r="K19">
         <v>0</v>
       </c>
       <c r="L19">
-        <v>3.3899999999999998E-3</v>
+        <v>4.7739999999999996E-3</v>
       </c>
       <c r="M19">
-        <v>0</v>
+        <v>9.5500000000000001E-4</v>
       </c>
       <c r="N19">
         <v>0</v>
@@ -2107,25 +2107,25 @@
         <v>0</v>
       </c>
       <c r="Q19">
-        <v>0.16041900000000001</v>
+        <v>0.114273</v>
       </c>
       <c r="R19">
-        <v>3.2490000000000002E-3</v>
+        <v>2.745E-3</v>
       </c>
       <c r="S19">
-        <v>0.63586600000000004</v>
+        <v>0.64132400000000001</v>
       </c>
       <c r="T19">
-        <v>5.6979999999999999E-3</v>
+        <v>7.7039999999999999E-3</v>
       </c>
       <c r="U19">
-        <v>1.14E-3</v>
+        <v>9.6299999999999999E-4</v>
       </c>
       <c r="V19">
-        <v>5.6979999999999999E-3</v>
+        <v>6.7409999999999996E-3</v>
       </c>
       <c r="W19">
-        <v>1.14E-3</v>
+        <v>2.8890000000000001E-3</v>
       </c>
       <c r="X19">
         <v>0</v>
@@ -2134,13 +2134,13 @@
         <v>0</v>
       </c>
       <c r="Z19">
-        <v>9.2302999999999996E-2</v>
+        <v>9.9183999999999994E-2</v>
       </c>
       <c r="AA19">
         <v>0</v>
       </c>
       <c r="AB19">
-        <v>0</v>
+        <v>9.6299999999999999E-4</v>
       </c>
       <c r="AC19">
         <v>0</v>
@@ -2149,7 +2149,7 @@
         <v>0</v>
       </c>
       <c r="AE19">
-        <v>5.237E-2</v>
+        <v>6.0624999999999998E-2</v>
       </c>
     </row>
     <row r="20" spans="1:31" x14ac:dyDescent="0.45">
@@ -2160,31 +2160,31 @@
         <v>0</v>
       </c>
       <c r="C20">
-        <v>2.5392000000000001E-2</v>
+        <v>2.2685E-2</v>
       </c>
       <c r="D20">
         <v>0</v>
       </c>
       <c r="E20">
-        <v>4.0439999999999999E-3</v>
+        <v>1.2467000000000001E-2</v>
       </c>
       <c r="F20">
         <v>0</v>
       </c>
       <c r="G20">
-        <v>1.2132E-2</v>
+        <v>9.3500000000000007E-3</v>
       </c>
       <c r="H20">
         <v>0</v>
       </c>
       <c r="I20">
-        <v>8.0879999999999997E-3</v>
+        <v>9.3500000000000007E-3</v>
       </c>
       <c r="J20">
         <v>0</v>
       </c>
       <c r="K20">
-        <v>4.0439999999999999E-3</v>
+        <v>3.117E-3</v>
       </c>
       <c r="L20">
         <v>0</v>
@@ -2202,7 +2202,7 @@
         <v>0</v>
       </c>
       <c r="Q20">
-        <v>0</v>
+        <v>3.143E-3</v>
       </c>
       <c r="R20">
         <v>0</v>
@@ -2211,16 +2211,16 @@
         <v>0</v>
       </c>
       <c r="T20">
-        <v>0.73419699999999999</v>
+        <v>0.70413000000000003</v>
       </c>
       <c r="U20">
         <v>0</v>
       </c>
       <c r="V20">
-        <v>0.19170699999999999</v>
+        <v>0.20746700000000001</v>
       </c>
       <c r="W20">
-        <v>0</v>
+        <v>3.143E-3</v>
       </c>
       <c r="X20">
         <v>0</v>
@@ -2232,7 +2232,7 @@
         <v>0</v>
       </c>
       <c r="AA20">
-        <v>1.6315E-2</v>
+        <v>1.2574E-2</v>
       </c>
       <c r="AB20">
         <v>0</v>
@@ -2244,7 +2244,7 @@
         <v>0</v>
       </c>
       <c r="AE20">
-        <v>4.0790000000000002E-3</v>
+        <v>1.2574E-2</v>
       </c>
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.45">
@@ -2258,19 +2258,19 @@
         <v>0</v>
       </c>
       <c r="D21">
-        <v>2.6162999999999999E-2</v>
+        <v>2.0076E-2</v>
       </c>
       <c r="E21">
         <v>0</v>
       </c>
       <c r="F21">
-        <v>3.9245000000000002E-2</v>
+        <v>4.0150999999999999E-2</v>
       </c>
       <c r="G21">
         <v>0</v>
       </c>
       <c r="H21">
-        <v>1.3082E-2</v>
+        <v>1.0038E-2</v>
       </c>
       <c r="I21">
         <v>0</v>
@@ -2297,25 +2297,25 @@
         <v>0</v>
       </c>
       <c r="Q21">
-        <v>3.7613000000000001E-2</v>
+        <v>2.8861000000000001E-2</v>
       </c>
       <c r="R21">
         <v>0</v>
       </c>
       <c r="S21">
-        <v>1.3194000000000001E-2</v>
+        <v>2.0247999999999999E-2</v>
       </c>
       <c r="T21">
-        <v>1.3194000000000001E-2</v>
+        <v>1.0123999999999999E-2</v>
       </c>
       <c r="U21">
-        <v>0.35624299999999998</v>
+        <v>0.334096</v>
       </c>
       <c r="V21">
         <v>0</v>
       </c>
       <c r="W21">
-        <v>0.422213</v>
+        <v>0.43533699999999997</v>
       </c>
       <c r="X21">
         <v>0</v>
@@ -2339,7 +2339,7 @@
         <v>0</v>
       </c>
       <c r="AE21">
-        <v>7.9052999999999998E-2</v>
+        <v>0.10106900000000001</v>
       </c>
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.45">
@@ -2368,7 +2368,7 @@
         <v>0</v>
       </c>
       <c r="I22">
-        <v>6.2E-2</v>
+        <v>9.9232000000000001E-2</v>
       </c>
       <c r="J22">
         <v>0</v>
@@ -2401,13 +2401,13 @@
         <v>0</v>
       </c>
       <c r="T22">
-        <v>0.18759999999999999</v>
+        <v>0.10008499999999999</v>
       </c>
       <c r="U22">
         <v>0</v>
       </c>
       <c r="V22">
-        <v>0.43773299999999998</v>
+        <v>0.60051200000000005</v>
       </c>
       <c r="W22">
         <v>0</v>
@@ -2422,7 +2422,7 @@
         <v>0</v>
       </c>
       <c r="AA22">
-        <v>0.25013299999999999</v>
+        <v>0.15012800000000001</v>
       </c>
       <c r="AB22">
         <v>0</v>
@@ -2434,7 +2434,7 @@
         <v>0</v>
       </c>
       <c r="AE22">
-        <v>6.2533000000000005E-2</v>
+        <v>5.0042999999999997E-2</v>
       </c>
     </row>
     <row r="23" spans="1:31" x14ac:dyDescent="0.45">
@@ -2454,7 +2454,7 @@
         <v>0</v>
       </c>
       <c r="F23">
-        <v>0.19863400000000001</v>
+        <v>0.16548099999999999</v>
       </c>
       <c r="G23">
         <v>0</v>
@@ -2505,7 +2505,7 @@
         <v>0</v>
       </c>
       <c r="W23">
-        <v>0.20034099999999999</v>
+        <v>0.33380700000000002</v>
       </c>
       <c r="X23">
         <v>0</v>
@@ -2529,7 +2529,7 @@
         <v>0</v>
       </c>
       <c r="AE23">
-        <v>0.601024</v>
+        <v>0.50071100000000002</v>
       </c>
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.45">
@@ -2635,13 +2635,13 @@
         <v>0</v>
       </c>
       <c r="C25">
-        <v>3.0896E-2</v>
+        <v>3.6394999999999997E-2</v>
       </c>
       <c r="D25">
         <v>0</v>
       </c>
       <c r="E25">
-        <v>9.2688999999999994E-2</v>
+        <v>0.10918600000000001</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -2674,13 +2674,13 @@
         <v>0</v>
       </c>
       <c r="P25">
-        <v>1.7840000000000002E-2</v>
+        <v>0</v>
       </c>
       <c r="Q25">
         <v>0</v>
       </c>
       <c r="R25">
-        <v>0.29766100000000001</v>
+        <v>0.24873600000000001</v>
       </c>
       <c r="S25">
         <v>0</v>
@@ -2701,7 +2701,7 @@
         <v>0</v>
       </c>
       <c r="Y25">
-        <v>0.24929499999999999</v>
+        <v>0.29366500000000001</v>
       </c>
       <c r="Z25">
         <v>0</v>
@@ -2719,7 +2719,7 @@
         <v>0</v>
       </c>
       <c r="AE25">
-        <v>0.31161899999999998</v>
+        <v>0.31201899999999999</v>
       </c>
     </row>
     <row r="26" spans="1:31" x14ac:dyDescent="0.45">
@@ -2739,7 +2739,7 @@
         <v>0</v>
       </c>
       <c r="F26">
-        <v>0.106327</v>
+        <v>3.2001000000000002E-2</v>
       </c>
       <c r="G26">
         <v>0</v>
@@ -2757,7 +2757,7 @@
         <v>0</v>
       </c>
       <c r="L26">
-        <v>0</v>
+        <v>3.2001000000000002E-2</v>
       </c>
       <c r="M26">
         <v>0</v>
@@ -2772,13 +2772,13 @@
         <v>0</v>
       </c>
       <c r="Q26">
-        <v>7.1494000000000002E-2</v>
+        <v>6.4551999999999998E-2</v>
       </c>
       <c r="R26">
         <v>0</v>
       </c>
       <c r="S26">
-        <v>0.28597499999999998</v>
+        <v>0.32275799999999999</v>
       </c>
       <c r="T26">
         <v>0</v>
@@ -2787,10 +2787,10 @@
         <v>0</v>
       </c>
       <c r="V26">
-        <v>0</v>
+        <v>3.2275999999999999E-2</v>
       </c>
       <c r="W26">
-        <v>3.5747000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="X26">
         <v>0</v>
@@ -2799,7 +2799,7 @@
         <v>0</v>
       </c>
       <c r="Z26">
-        <v>0.25022800000000001</v>
+        <v>0.25820599999999999</v>
       </c>
       <c r="AA26">
         <v>0</v>
@@ -2814,7 +2814,7 @@
         <v>0</v>
       </c>
       <c r="AE26">
-        <v>0.25022800000000001</v>
+        <v>0.25820599999999999</v>
       </c>
     </row>
     <row r="27" spans="1:31" x14ac:dyDescent="0.45">
@@ -2953,7 +2953,7 @@
         <v>0</v>
       </c>
       <c r="N28">
-        <v>5.2229999999999999E-2</v>
+        <v>3.9685999999999999E-2</v>
       </c>
       <c r="O28">
         <v>0</v>
@@ -2977,7 +2977,7 @@
         <v>0</v>
       </c>
       <c r="V28">
-        <v>5.2678999999999997E-2</v>
+        <v>4.0027E-2</v>
       </c>
       <c r="W28">
         <v>0</v>
@@ -2995,7 +2995,7 @@
         <v>0</v>
       </c>
       <c r="AB28">
-        <v>0.79018200000000005</v>
+        <v>0.84057300000000001</v>
       </c>
       <c r="AC28">
         <v>0</v>
@@ -3004,7 +3004,7 @@
         <v>0</v>
       </c>
       <c r="AE28">
-        <v>0.104909</v>
+        <v>7.9713000000000006E-2</v>
       </c>
     </row>
     <row r="29" spans="1:31" x14ac:dyDescent="0.45">
@@ -3093,13 +3093,13 @@
         <v>0</v>
       </c>
       <c r="AC29">
-        <v>0</v>
+        <v>0.50214000000000003</v>
       </c>
       <c r="AD29">
         <v>0</v>
       </c>
       <c r="AE29">
-        <v>1</v>
+        <v>0.49786000000000002</v>
       </c>
     </row>
     <row r="30" spans="1:31" x14ac:dyDescent="0.45">

</xml_diff>